<commit_message>
additions for mantle classification scheme
</commit_message>
<xml_diff>
--- a/pide/pide_src/geochem/Average_Composition_GEOROC.xlsx
+++ b/pide/pide_src/geochem/Average_Composition_GEOROC.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="33">
   <si>
     <t xml:space="preserve">Alkali-Basalt</t>
   </si>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t xml:space="preserve">TOT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NA2O/K2O</t>
   </si>
   <si>
     <t xml:space="preserve">Basaltic-Trachyandesite</t>
@@ -227,8 +230,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N84"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:O84"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -278,6 +281,9 @@
       <c r="N2" s="2" t="s">
         <v>14</v>
       </c>
+      <c r="O2" s="0" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="n">
@@ -323,6 +329,10 @@
         <f aca="false">SUM(A3:M3)</f>
         <v>99.1277715242117</v>
       </c>
+      <c r="O3" s="0" t="n">
+        <f aca="false">K3/J3</f>
+        <v>2.31111864551799</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="n">
@@ -368,10 +378,14 @@
         <f aca="false">SUM(A4:M4)</f>
         <v>100</v>
       </c>
+      <c r="O4" s="0" t="n">
+        <f aca="false">K4/J4</f>
+        <v>2.31111864551799</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -462,6 +476,10 @@
         <f aca="false">SUM(A8:M8)</f>
         <v>98.4237999224418</v>
       </c>
+      <c r="O8" s="0" t="n">
+        <f aca="false">K8/J8</f>
+        <v>1.43486643343205</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="n">
@@ -507,10 +525,14 @@
         <f aca="false">SUM(A9:M9)</f>
         <v>100</v>
       </c>
+      <c r="O9" s="0" t="n">
+        <f aca="false">K9/J9</f>
+        <v>1.43486643343205</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -601,6 +623,10 @@
         <f aca="false">SUM(A13:M13)</f>
         <v>97.5749087163126</v>
       </c>
+      <c r="O13" s="0" t="n">
+        <f aca="false">K13/J13</f>
+        <v>1.37794003727392</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="n">
@@ -646,10 +672,14 @@
         <f aca="false">SUM(A14:M14)</f>
         <v>100</v>
       </c>
+      <c r="O14" s="0" t="n">
+        <f aca="false">K14/J14</f>
+        <v>1.37794003727392</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -740,6 +770,10 @@
         <f aca="false">SUM(A18:M18)</f>
         <v>98.8165647109027</v>
       </c>
+      <c r="O18" s="0" t="n">
+        <f aca="false">K18/J18</f>
+        <v>1.25533052167074</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="n">
@@ -785,10 +819,14 @@
         <f aca="false">SUM(A19:M19)</f>
         <v>100</v>
       </c>
+      <c r="O19" s="0" t="n">
+        <f aca="false">K19/J19</f>
+        <v>1.25533052167074</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -879,6 +917,10 @@
         <f aca="false">SUM(A23:M23)</f>
         <v>99.023141560708</v>
       </c>
+      <c r="O23" s="0" t="n">
+        <f aca="false">K23/J23</f>
+        <v>0.85944442974702</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="n">
@@ -924,10 +966,14 @@
         <f aca="false">SUM(A24:M24)</f>
         <v>100</v>
       </c>
+      <c r="O24" s="0" t="n">
+        <f aca="false">K24/J24</f>
+        <v>0.859444429747022</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1018,6 +1064,10 @@
         <f aca="false">SUM(A28:M28)</f>
         <v>99.289196776028</v>
       </c>
+      <c r="O28" s="0" t="n">
+        <f aca="false">K28/J28</f>
+        <v>2.26645828057185</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="n">
@@ -1063,10 +1113,14 @@
         <f aca="false">SUM(A29:M29)</f>
         <v>100</v>
       </c>
+      <c r="O29" s="0" t="n">
+        <f aca="false">K29/J29</f>
+        <v>2.26645828057184</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1157,6 +1211,10 @@
         <f aca="false">SUM(A33:M33)</f>
         <v>99.0319850605406</v>
       </c>
+      <c r="O33" s="0" t="n">
+        <f aca="false">K33/J33</f>
+        <v>1.21247049614282</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="n">
@@ -1202,10 +1260,14 @@
         <f aca="false">SUM(A34:M34)</f>
         <v>100</v>
       </c>
+      <c r="O34" s="0" t="n">
+        <f aca="false">K34/J34</f>
+        <v>1.21247049614282</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1296,6 +1358,10 @@
         <f aca="false">SUM(A38:M38)</f>
         <v>98.9368704317937</v>
       </c>
+      <c r="O38" s="0" t="n">
+        <f aca="false">K38/J38</f>
+        <v>0.703772973337105</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="n">
@@ -1341,10 +1407,14 @@
         <f aca="false">SUM(A39:M39)</f>
         <v>100</v>
       </c>
+      <c r="O39" s="0" t="n">
+        <f aca="false">K39/J39</f>
+        <v>0.703772973337106</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1435,6 +1505,10 @@
         <f aca="false">SUM(A43:M43)</f>
         <v>98.6701625624853</v>
       </c>
+      <c r="O43" s="0" t="n">
+        <f aca="false">K43/J43</f>
+        <v>1.19997788225922</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="n">
@@ -1480,10 +1554,14 @@
         <f aca="false">SUM(A44:M44)</f>
         <v>100</v>
       </c>
+      <c r="O44" s="0" t="n">
+        <f aca="false">K44/J44</f>
+        <v>1.19997788225922</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1574,6 +1652,10 @@
         <f aca="false">SUM(A48:M48)</f>
         <v>99.6768302055768</v>
       </c>
+      <c r="O48" s="0" t="n">
+        <f aca="false">K48/J48</f>
+        <v>1.01246947517441</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="n">
@@ -1619,10 +1701,14 @@
         <f aca="false">SUM(A49:M49)</f>
         <v>100</v>
       </c>
+      <c r="O49" s="0" t="n">
+        <f aca="false">K49/J49</f>
+        <v>1.01246947517441</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1713,6 +1799,10 @@
         <f aca="false">SUM(A53:M53)</f>
         <v>99.3051013536608</v>
       </c>
+      <c r="O53" s="0" t="n">
+        <f aca="false">K53/J53</f>
+        <v>2.51889560627012</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="n">
@@ -1758,10 +1848,14 @@
         <f aca="false">SUM(A54:M54)</f>
         <v>100</v>
       </c>
+      <c r="O54" s="0" t="n">
+        <f aca="false">K54/J54</f>
+        <v>2.51889560627013</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1852,6 +1946,10 @@
         <f aca="false">SUM(A58:M58)</f>
         <v>99.514964374541</v>
       </c>
+      <c r="O58" s="0" t="n">
+        <f aca="false">K58/J58</f>
+        <v>1.50878811028387</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="n">
@@ -1897,10 +1995,14 @@
         <f aca="false">SUM(A59:M59)</f>
         <v>100</v>
       </c>
+      <c r="O59" s="0" t="n">
+        <f aca="false">K59/J59</f>
+        <v>1.50878811028387</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1991,6 +2093,10 @@
         <f aca="false">SUM(A63:M63)</f>
         <v>98.9703632009943</v>
       </c>
+      <c r="O63" s="0" t="n">
+        <f aca="false">K63/J63</f>
+        <v>2.85122959544664</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="n">
@@ -2036,10 +2142,14 @@
         <f aca="false">SUM(A64:M64)</f>
         <v>100</v>
       </c>
+      <c r="O64" s="0" t="n">
+        <f aca="false">K64/J64</f>
+        <v>2.85122959544664</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2130,6 +2240,10 @@
         <f aca="false">SUM(A68:M68)</f>
         <v>99.540151225395</v>
       </c>
+      <c r="O68" s="0" t="n">
+        <f aca="false">K68/J68</f>
+        <v>1.99922350054169</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="n">
@@ -2175,10 +2289,14 @@
         <f aca="false">SUM(A69:M69)</f>
         <v>100</v>
       </c>
+      <c r="O69" s="0" t="n">
+        <f aca="false">K69/J69</f>
+        <v>1.9992235005417</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2195,7 +2313,7 @@
         <v>4</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F72" s="2" t="s">
         <v>6</v>
@@ -2269,6 +2387,10 @@
         <f aca="false">SUM(A73:M73)</f>
         <v>99.6538700487595</v>
       </c>
+      <c r="O73" s="0" t="n">
+        <f aca="false">K73/J73</f>
+        <v>0.798459652862628</v>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="n">
@@ -2314,10 +2436,14 @@
         <f aca="false">SUM(A74:M74)</f>
         <v>100</v>
       </c>
+      <c r="O74" s="0" t="n">
+        <f aca="false">K74/J74</f>
+        <v>0.798459652862627</v>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2408,6 +2534,10 @@
         <f aca="false">SUM(A78:M78)</f>
         <v>99.2789526924704</v>
       </c>
+      <c r="O78" s="0" t="n">
+        <f aca="false">K78/J78</f>
+        <v>1.48803999047123</v>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="0" t="n">
@@ -2453,10 +2583,14 @@
         <f aca="false">SUM(A79:M79)</f>
         <v>100</v>
       </c>
+      <c r="O79" s="0" t="n">
+        <f aca="false">K79/J79</f>
+        <v>1.48803999047122</v>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2547,6 +2681,10 @@
         <f aca="false">SUM(A83:M83)</f>
         <v>99.1202705748191</v>
       </c>
+      <c r="O83" s="0" t="n">
+        <f aca="false">K83/J83</f>
+        <v>0.983856853169132</v>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="0" t="n">
@@ -2591,6 +2729,10 @@
       <c r="N84" s="2" t="n">
         <f aca="false">SUM(A84:M84)</f>
         <v>100</v>
+      </c>
+      <c r="O84" s="0" t="n">
+        <f aca="false">K84/J84</f>
+        <v>0.983856853169132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>